<commit_message>
Multi-member dashboard: per-member FEC/SOD data, FD disclosure, vendor categories
- Generalize dashboards/index.html to one template that loads any member by
  ?member=<bioguide> (entities, identity, charts, flags all data-driven).
- build/build_member.py: resolve candidate->committee, pull FEC Schedule B + SOD
  office spending per member, FEC-cross-checked against official totals.
- build/fd_parser.py + add_disclosure.py: parse House Financial Disclosure PDFs
  (pdfplumber) into structured assets/liabilities/income/transactions; render in
  the Financial Disclosure tab with a source-PDF link.
- Vendor Intelligence rebuilt from each member's own disbursements (by_category
  over all rows); Swalwell-only deep-dives hidden for other members.
- Member data lives under dashboards/members/ so GitHub Pages serves it.
- 9 sample members built (Swalwell dashboard unchanged); expandable via the manifest.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master/119th_MASTER_LIST.xlsx
+++ b/data/master/119th_MASTER_LIST.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amandakoski/Documents/Claude/Projects/Dashboard Homepage/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amandakoski/Documents/Claude/Suffrage and Sass/Sovereign AI/data/master/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFAEF68-07D2-DD46-A71C-2E6116B1E776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28999F08-D352-484B-A553-8BB176269F32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="600" windowWidth="33720" windowHeight="19160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24766,7 +24766,9 @@
       </c>
     </row>
     <row r="24" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A24" s="2"/>
+      <c r="A24" s="2">
+        <v>2</v>
+      </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
         <v>420</v>
@@ -25935,7 +25937,9 @@
       </c>
     </row>
     <row r="37" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
+      <c r="A37" s="3">
+        <v>3</v>
+      </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3" t="s">
         <v>186</v>
@@ -34447,7 +34451,9 @@
       </c>
     </row>
     <row r="131" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A131" s="3"/>
+      <c r="A131" s="3">
+        <v>4</v>
+      </c>
       <c r="B131" s="3"/>
       <c r="C131" s="3" t="s">
         <v>256</v>
@@ -58042,7 +58048,9 @@
       </c>
     </row>
     <row r="390" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A390" s="2"/>
+      <c r="A390" s="2">
+        <v>5</v>
+      </c>
       <c r="B390" s="2"/>
       <c r="C390" s="2" t="s">
         <v>6525</v>

</xml_diff>